<commit_message>
Added examples for sine environment, sdynpy frf, exodus, and state space virtual hardware.
</commit_message>
<xml_diff>
--- a/src/rattlesnake/examples/hardware/sdynpy_frf/sdynpy_frf_v3.xlsx
+++ b/src/rattlesnake/examples/hardware/sdynpy_frf/sdynpy_frf_v3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmlangs\Desktop\examples\hardware\sdynpy_frf\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmlangs\Desktop\rattlesnake-vibration-controller-headless\src\rattlesnake\examples\hardware\sdynpy_frf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAC0656E-CFF3-4C77-8469-E273A90073A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1126ADC5-B144-4F3B-964D-328EC83388D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6070" yWindow="1960" windowWidth="28790" windowHeight="15350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Channel Table" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="61">
   <si>
     <t>Test Article Definition</t>
   </si>
@@ -204,9 +204,6 @@
   </si>
   <si>
     <t>135</t>
-  </si>
-  <si>
-    <t>C:\Users\cmlangs\Desktop\rattlesnake-vibration-controller-headless\src\rattlesnake\examples/hardware/sdynpy_frf/sdynpy_frf.npz</t>
   </si>
 </sst>
 </file>
@@ -1138,9 +1135,6 @@
       <c r="A2" t="s">
         <v>28</v>
       </c>
-      <c r="B2" t="s">
-        <v>61</v>
-      </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">

</xml_diff>